<commit_message>
Fluxo de caixa: alerta de exposição, gráfico novo e cards em uma linha
- Aba Fluxo de caixa mostra só o Andrade Home Resort
- Sete indicadores compactos na mesma linha, gráfico logo abaixo
- Alerta com o mês em que o caixa acumulado fica negativo
- Colunas sólidas com rótulos e linhas acumuladas com área preenchida
- Planilhas de vendas e cadastro atualizadas

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Cadastro de Unidades.xlsx
+++ b/Cadastro de Unidades.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\filip\OneDrive\Área de Trabalho\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\filip\OneDrive\Área de Trabalho\SALES DASHBOARD - CLAUDE\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7CF13EC-AAB0-430B-8058-8DA233E47A7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cadastro de Unidades" sheetId="2" r:id="rId1"/>

</xml_diff>